<commit_message>
Updated PED version history and Decision log ID conflict
updated the PED to use proper formatted versions and also fixed the decision log error that was showing 2 separate decision 7 logs... Updated to reflect consistency.
</commit_message>
<xml_diff>
--- a/docs/decisions/Decision Log/Decision Log v0.4.xlsx
+++ b/docs/decisions/Decision Log/Decision Log v0.4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4c906530d9ff38bc/Desktop/SEN381/Ticketing-System/docs/decisions/Decision Log/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="211" documentId="8_{DA8A1402-F87E-4E16-A5E2-7754A6675A1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD37A5A6-2B21-4DD4-BF73-84E0249273A8}"/>
+  <xr:revisionPtr revIDLastSave="286" documentId="8_{DA8A1402-F87E-4E16-A5E2-7754A6675A1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A77F1E8-432F-4BA0-9F27-6829C9386ABD}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{C10860F7-7028-4DF0-9A0A-0CD539FC6C60}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="89">
   <si>
     <t>Decision Log</t>
   </si>
@@ -173,9 +173,6 @@
     <t>Ethan</t>
   </si>
   <si>
-    <t>2026/09/06  - Revised 2206/09/09</t>
-  </si>
-  <si>
     <t>Exclude a native mobile application from the committed scope; mobile access is delivered through responsive web</t>
   </si>
   <si>
@@ -185,9 +182,6 @@
     <t>Places a usability obligation on the web interface at mobile viewports, to be specified measurably by Member B under CON-005. Following the revision, the exclusion is no longer a team preference and cannot be revisited without a change request under Master Brief s.14. Reduces the risk that scope pressure later reopens the question.</t>
   </si>
   <si>
-    <t>DEC-007 (Revised)</t>
-  </si>
-  <si>
     <t>DEC-009</t>
   </si>
   <si>
@@ -288,13 +282,37 @@
   </si>
   <si>
     <t>Publish a domain event from the status-transition service and let interested components subscribe to it, using in-process event publication within the application layer</t>
+  </si>
+  <si>
+    <t>Direct orchestration, in which the transition service invokes each consequence in sequence; distributed messaging through a broker or queue</t>
+  </si>
+  <si>
+    <t>A status transition produces several outcomes belonging to different parts of the system: the status change and its validation (FR-6.2, FR-6.4), the immutable history entry (FR-6.3, FR-6.7), in-application feedback to the requester (FR-3.4, SCP-004) and the counts the management view reads (feature group 8). CON-015 and NFR-1.9 place the audit write below the application layer through Atlas managed database triggers, which removes it from this decision rather than solving it here. The remaining consequence set is known to be incomplete: SCP-014 is deferred rather than excluded and its dependency on DEC-003 has closed, so a further consequence is anticipated. Under direct orchestration, admitting SCP-014 later means editing transition code already reviewed under DEC-008 and verified against its acceptance criteria, converting a scope decision into a regression risk. Assignment 2 s.2.5 compared the two approaches across coupling, cohesion, layering, extensibility, testability and misuse risk. Gamma et al. (1994) record that the coupling between subject and observer is abstract and minimal and permits the two to occupy different layers, which aligns with CON-012 and NFR-1.7 rather than working against them. EventEmitter ships with the runtime selected under DEC-002, so no dependency is added against CON-003 or CON-008. Distributed messaging was rejected as disproportionate: it would introduce a network boundary and a third external provider for a consequence set of two.</t>
+  </si>
+  <si>
+    <t>SCP-014 attaches as a new subscriber rather than as an edit to verified code. The transition becomes testable by asserting publication rather than by constructing every collaborator. Three costs are accepted and recorded. No single location states what a transition does, which cuts against RSK-012; all subscriptions are therefore registered in one module so the set is enumerable by reading one file. EventEmitter dispatches synchronously, so a subscriber that throws would propagate the error back into the transition that published the event; subscriber invocation is wrapped so errors are logged and contained, and the transition and its consequences are deliberately not atomic with one another. Subscriber ordering is not guaranteed meaningful, so no consequence may depend on another having run. Affects FR-3.4, FR-6.2, FR-6.3, FR-6.4, FR-6.7, NFR-1.7, NFR-1.9, SCP-004, SCP-008, SCP-014; a component diagram is required.</t>
+  </si>
+  <si>
+    <t>Enforce authorisation at three points against one documented rule set: composed Express middleware at the route boundary for function-level access, the service layer for object-level access once the request document is loaded, and the response serialiser for field-level access.</t>
+  </si>
+  <si>
+    <t>A single protection proxy per service; a centralised policy service called from every entry point; an explicit guard call at the top of each service method</t>
+  </si>
+  <si>
+    <t>NFR-3.3 requires every authorisation rule to be enforced at the server on each request at every entry point, including endpoints not reachable through the interface, and CON-019 rules out treating a hidden interface control as an access restriction. DEC-004 records role-based access control as architecturally significant. The requirement set is not uniform: function-level access (FR-1.3, FR-6.4), object-level access depending on the request rather than the caller (FR-3.6, FR-4.1), and field-level access for security-category requests under the CFL-002 resolution (FR-1.5, FR-3.5, FR-8.6, NFR-4.4). Assignment 2 s.2.6 compared three approaches and deliberately held the recommendation open, recording the guard-call option as defensible under CON-004 and noting that a hybrid had not been researched. DEC-002 has since selected Express, whose middleware is a protection proxy in the idiom of the runtime: it stands in front of the handler, shares the request and response interface, and either forwards or refuses. Adopting it is the Assignment 2 recommendation expressed in the committed technology rather than a departure from it. The hybrid follows from the three granularities: the middleware chain runs before the document is fetched, so an object-level check cannot be made there. The guard-call alternative is rejected on detectability, which was the deciding criterion in Assignment 2 s.2.6.3: a missing guard call is invisible, whereas a route registered without its guard is visible in the route table and can be asserted against automatically, which is what CON-019 adversarial testing needs.</t>
+  </si>
+  <si>
+    <t>Enforcement is distributed across three locations while the rule set remains single, which is more to hold in mind and more to check in review. Middleware ordering is load-bearing and fails silently when wrong, so authentication and authorisation are composed as one named guard rather than registered separately per route. A route registered without its guard is permitted by default, mitigated by an automated assertion over the route table that every non-public route carries it; that assertion is the evidence NFR-3.3 requires. The rule the serialiser enforces rests on CFL-002, which remains Proposed and unconfirmed with STK-006, so this decision would require revision if the resolution is not agreed; condition C-01 remains open and the exposure is tracked as RSK-009. Affects FR-1.3, FR-1.5, FR-1.6, FR-3.5, FR-3.6, FR-4.1, FR-6.4, FR-8.6, NFR-3.3, NFR-4.4, SCP-005, SCP-012; a sequence diagram showing both refusal points is required.</t>
+  </si>
+  <si>
+    <t>DEC-013</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -359,14 +377,6 @@
     </font>
     <font>
       <sz val="8"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -465,7 +475,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -515,35 +525,29 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -558,17 +562,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
-    <dxf>
-      <font>
-        <color rgb="FFA6A6A6"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFA6A6A6"/>
-      </font>
-    </dxf>
+  <dxfs count="17">
     <dxf>
       <font>
         <color rgb="FFA6A6A6"/>
@@ -616,6 +610,56 @@
         <color rgb="FFA6A6A6"/>
       </font>
     </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFA6A6A6"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFA6A6A6"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFA6A6A6"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFA6A6A6"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFA6A6A6"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFA6A6A6"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFA6A6A6"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFA6A6A6"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFA6A6A6"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFA6A6A6"/>
+      </font>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -632,6 +676,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -970,32 +1018,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="25.8" x14ac:dyDescent="0.3">
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
     </row>
     <row r="2" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B2" s="26" t="s">
-        <v>78</v>
-      </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
+      <c r="B2" s="22" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="21"/>
     </row>
     <row r="4" spans="2:16" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
@@ -1023,16 +1071,16 @@
         <v>8</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="N4" s="23" t="s">
+      <c r="N4" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="O4" s="23"/>
-      <c r="P4" s="23"/>
+      <c r="O4" s="24"/>
+      <c r="P4" s="24"/>
     </row>
     <row r="5" spans="2:16" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
@@ -1054,23 +1102,25 @@
       <c r="G5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="6" t="s">
         <v>15</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="J5" s="17"/>
+      <c r="J5" s="6" t="s">
+        <v>15</v>
+      </c>
       <c r="K5" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="N5" s="27" t="s">
+      <c r="N5" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="O5" s="27"/>
+      <c r="O5" s="25"/>
       <c r="P5" s="13">
-        <f>COUNTIF($K$5:$K$149,"DECIDED")</f>
-        <v>10</v>
+        <f>COUNTIF($K$5:$K$148,"DECIDED")</f>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="2:16" ht="201.6" x14ac:dyDescent="0.3">
@@ -1082,35 +1132,35 @@
         <v>46294</v>
       </c>
       <c r="D6" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="G6" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="E6" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="11" t="s">
         <v>15</v>
       </c>
       <c r="I6" s="11" t="s">
         <v>43</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="N6" s="27" t="s">
-        <v>73</v>
-      </c>
-      <c r="O6" s="27"/>
+      <c r="N6" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="O6" s="25"/>
       <c r="P6" s="13">
-        <f>COUNTIF($K$5:$K$15,"DEFERRED")</f>
+        <f>COUNTIF($K$5:$K$513,"DEFERRED")</f>
         <v>1</v>
       </c>
     </row>
@@ -1123,35 +1173,35 @@
         <v>46294</v>
       </c>
       <c r="D7" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="E7" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="6" t="s">
         <v>15</v>
       </c>
       <c r="I7" s="6" t="s">
         <v>43</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K7" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="N7" s="28" t="s">
-        <v>75</v>
-      </c>
-      <c r="O7" s="29"/>
+      <c r="N7" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="O7" s="27"/>
       <c r="P7" s="13">
-        <f>COUNTIF($K$5:$K$12,"SUPERSEDED")</f>
+        <f>COUNTIF($K$5:$K$762,"SUPERSEDED")</f>
         <v>1</v>
       </c>
     </row>
@@ -1175,23 +1225,25 @@
       <c r="G8" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" s="11" t="s">
         <v>15</v>
       </c>
       <c r="I8" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="J8" s="11"/>
+      <c r="J8" s="11" t="s">
+        <v>15</v>
+      </c>
       <c r="K8" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="N8" s="22" t="s">
+      <c r="N8" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="O8" s="22"/>
+      <c r="O8" s="23"/>
       <c r="P8" s="14">
         <f>SUM(P5:P7)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="2:16" ht="158.4" x14ac:dyDescent="0.3">
@@ -1203,25 +1255,25 @@
         <v>46294</v>
       </c>
       <c r="D9" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="6" t="s">
         <v>15</v>
       </c>
       <c r="I9" s="6" t="s">
         <v>43</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K9" s="12" t="s">
         <v>16</v>
@@ -1247,13 +1299,15 @@
       <c r="G10" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="11" t="s">
         <v>15</v>
       </c>
       <c r="I10" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="J10" s="11"/>
+      <c r="J10" s="11" t="s">
+        <v>15</v>
+      </c>
       <c r="K10" s="12" t="s">
         <v>16</v>
       </c>
@@ -1278,15 +1332,17 @@
       <c r="G11" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="H11" s="6" t="s">
         <v>15</v>
       </c>
       <c r="I11" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="J11" s="6"/>
-      <c r="K11" s="21" t="s">
-        <v>74</v>
+      <c r="J11" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="K11" s="19" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="2:16" ht="72" x14ac:dyDescent="0.3">
@@ -1309,148 +1365,183 @@
       <c r="G12" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="10" t="s">
+      <c r="H12" s="11" t="s">
         <v>15</v>
       </c>
       <c r="I12" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="J12" s="11"/>
+      <c r="J12" s="11" t="s">
+        <v>15</v>
+      </c>
       <c r="K12" s="12" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="2:16" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="F13" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="G13" s="15" t="s">
+    <row r="13" spans="2:16" ht="160.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="H13" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="J13" s="6"/>
-      <c r="K13" s="7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" spans="2:16" ht="160.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C14" s="9">
+      <c r="C13" s="9">
         <f>DATE(2026,9,9)</f>
         <v>46274</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D13" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="F13" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="G13" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="F14" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="H14" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="I14" s="11" t="s">
+      <c r="H13" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="I13" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="J14" s="11"/>
-      <c r="K14" s="12" t="s">
+      <c r="J13" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="K13" s="12" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="2:16" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="B15" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="C15" s="16">
+    <row r="14" spans="2:16" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="B14" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" s="16">
         <f>DATE(2026,9,29)</f>
         <v>46294</v>
       </c>
-      <c r="D15" s="20" t="s">
+      <c r="D14" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="F14" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="E15" s="19" t="s">
+      <c r="G14" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="F15" s="19" t="s">
+      <c r="H14" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="G15" s="19" t="s">
+      <c r="I14" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="K14" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="H15" s="19" t="s">
-        <v>72</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="J15" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="K15" s="12" t="s">
-        <v>73</v>
-      </c>
     </row>
-    <row r="16" spans="2:16" ht="72" x14ac:dyDescent="0.3">
-      <c r="B16" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="C16" s="9">
+    <row r="15" spans="2:16" ht="302.39999999999998" x14ac:dyDescent="0.3">
+      <c r="B15" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C15" s="9">
         <f>DATE(2026,9,29)</f>
         <v>46294</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D15" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="F15" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11"/>
+      <c r="G15" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="H15" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="J15" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="K15" s="12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" spans="2:16" ht="316.8" x14ac:dyDescent="0.3">
+      <c r="B16" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C16" s="16">
+        <f>DATE(2026,9,29)</f>
+        <v>46294</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="F16" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="G16" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>15</v>
+      </c>
       <c r="K16" s="12" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B17" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="C17" s="16">
+    <row r="17" spans="2:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="C17" s="9">
         <f>DATE(2026,9,29)</f>
         <v>46294</v>
       </c>
-      <c r="D17" s="20"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="6"/>
-      <c r="J17" s="18"/>
-      <c r="K17" s="12"/>
+      <c r="D17" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="H17" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="I17" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="J17" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="K17" s="12" t="s">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1464,44 +1555,74 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="C5:C12">
-    <cfRule type="cellIs" dxfId="8" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="26" operator="equal">
       <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C14">
-    <cfRule type="cellIs" dxfId="7" priority="5" operator="equal">
+  <conditionalFormatting sqref="C13">
+    <cfRule type="cellIs" dxfId="15" priority="22" operator="equal">
       <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:H14">
-    <cfRule type="cellIs" dxfId="6" priority="8" operator="equal">
+  <conditionalFormatting sqref="C15">
+    <cfRule type="cellIs" dxfId="14" priority="19" operator="equal">
       <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J15">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
+  <conditionalFormatting sqref="H5">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="equal">
+      <formula>"—"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H7">
+    <cfRule type="cellIs" dxfId="12" priority="3" operator="equal">
+      <formula>"—"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H9">
+    <cfRule type="cellIs" dxfId="11" priority="4" operator="equal">
+      <formula>"—"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H11">
+    <cfRule type="cellIs" dxfId="10" priority="5" operator="equal">
+      <formula>"—"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H16">
+    <cfRule type="cellIs" dxfId="8" priority="7" operator="equal">
+      <formula>"—"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J5">
+    <cfRule type="cellIs" dxfId="7" priority="12" operator="equal">
+      <formula>"—"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J11">
+    <cfRule type="cellIs" dxfId="6" priority="11" operator="equal">
+      <formula>"—"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J14">
+    <cfRule type="cellIs" dxfId="4" priority="9" operator="equal">
+      <formula>"—"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J16">
+    <cfRule type="cellIs" dxfId="3" priority="8" operator="equal">
       <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K5:K17">
-    <cfRule type="containsText" dxfId="4" priority="6" operator="containsText" text="DECIDED">
+    <cfRule type="containsText" dxfId="2" priority="23" operator="containsText" text="DECIDED">
       <formula>NOT(ISERROR(SEARCH("DECIDED",K5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="7" operator="containsText" text="DEFERRED">
+    <cfRule type="containsText" dxfId="1" priority="24" operator="containsText" text="DEFERRED">
       <formula>NOT(ISERROR(SEARCH("DEFERRED",K5)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C16">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
-      <formula>"—"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H16">
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
-      <formula>"—"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J17">
+  <conditionalFormatting sqref="C17">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"—"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Add architecture baseline, diagrams and DEC-014 (#49)
Alternatives, layers, modules, tiers and DEC-014 ADR in PED §6A. Diagrams added; Decision Log updated. Refs #49
</commit_message>
<xml_diff>
--- a/docs/decisions/Decision Log/Decision Log v0.4.xlsx
+++ b/docs/decisions/Decision Log/Decision Log v0.4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4c906530d9ff38bc/Desktop/SEN381/Ticketing-System/docs/decisions/Decision Log/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cjbur\Desktop\New folder (2)\Ticketing-System\docs\decisions\Decision Log\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="286" documentId="8_{DA8A1402-F87E-4E16-A5E2-7754A6675A1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A77F1E8-432F-4BA0-9F27-6829C9386ABD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07F1E674-4044-4F89-B9EC-F690C62C3FB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{C10860F7-7028-4DF0-9A0A-0CD539FC6C60}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C10860F7-7028-4DF0-9A0A-0CD539FC6C60}"/>
   </bookViews>
   <sheets>
     <sheet name="Decision Log" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="95">
   <si>
     <t>Decision Log</t>
   </si>
@@ -306,6 +306,24 @@
   </si>
   <si>
     <t>DEC-013</t>
+  </si>
+  <si>
+    <t>DEC-014</t>
+  </si>
+  <si>
+    <t>Adopt a closed, layered modular monolith: three layers (presentation, application, data access) with downward single-boundary dependencies, divided into seven business-capability modules derived from the FR feature groups; lifecycle rules held as a framework-independent module inside the application layer; audit writes placed in the data store through database triggers.</t>
+  </si>
+  <si>
+    <t>Layered monolith organised by technical layer only; open or selectively open layering with a direct read path for reporting; service-based or microservices deployment.</t>
+  </si>
+  <si>
+    <t>CON-012 fixes the layered style and NFR-1.7 makes it testable, so the decision concerns boundaries and dependencies rather than style. The closed path protects ASR-01 (consistent authorisation) and ASR-02 (lifecycle integrity and audit). Business modules reduce collision between three part-time members (ASR-05, CON-004). One deployable unit fits CON-003 and CON-004 (ASR-06). Selectively open layering was rejected because NFR-1.7 forbids skipping a layer and a bypassed read path would skip the DEC-012 checks; the reporting performance need is met by the DEC-011 projection instead. Microservices were rejected: no requirement needs independent scaling or deployment, and distribution would split the single-transaction transition required by CON-017. Full record in PED §6A.8.</t>
+  </si>
+  <si>
+    <t>Pass-through code on simple reads (architecture sinkhole) accepted. No separate domain layer, so lifecycle rules depend on discipline to stay framework-free. One application instance is a single point of failure (RSK-017). Layer and module erosion under schedule pressure tracked as RSK-016. Repository structure must mirror the modules and layers (issue #51); the dependency rule is to be checked in CI (issue #52). A second application instance can be added without redesign because the application tier is stateless (ASR-04).</t>
+  </si>
+  <si>
+    <t>Christiaan</t>
   </si>
 </sst>
 </file>
@@ -562,12 +580,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
-    <dxf>
-      <font>
-        <color rgb="FFA6A6A6"/>
-      </font>
-    </dxf>
+  <dxfs count="14">
     <dxf>
       <font>
         <color rgb="FF7A3E00"/>
@@ -650,16 +663,6 @@
         <color rgb="FFA6A6A6"/>
       </font>
     </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFA6A6A6"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFA6A6A6"/>
-      </font>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -676,10 +679,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -999,25 +998,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51C17EC7-5E25-4DAF-A0FC-95E5CA365EC5}">
-  <dimension ref="B1:P17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B1:P18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.21875" customWidth="1"/>
-    <col min="2" max="2" width="18.109375" customWidth="1"/>
-    <col min="3" max="3" width="30.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.28515625" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" customWidth="1"/>
+    <col min="3" max="3" width="30.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="37" customWidth="1"/>
-    <col min="5" max="5" width="38.88671875" customWidth="1"/>
-    <col min="6" max="6" width="64.88671875" customWidth="1"/>
-    <col min="7" max="7" width="53.6640625" customWidth="1"/>
-    <col min="8" max="8" width="44.44140625" customWidth="1"/>
-    <col min="9" max="9" width="11.109375" customWidth="1"/>
-    <col min="10" max="10" width="46.21875" customWidth="1"/>
-    <col min="11" max="11" width="18.5546875" customWidth="1"/>
+    <col min="5" max="5" width="38.85546875" customWidth="1"/>
+    <col min="6" max="6" width="64.85546875" customWidth="1"/>
+    <col min="7" max="7" width="53.7109375" customWidth="1"/>
+    <col min="8" max="8" width="44.42578125" customWidth="1"/>
+    <col min="9" max="9" width="11.140625" customWidth="1"/>
+    <col min="10" max="10" width="46.28515625" customWidth="1"/>
+    <col min="11" max="11" width="18.5703125" customWidth="1"/>
     <col min="14" max="14" width="24" customWidth="1"/>
-    <col min="16" max="16" width="31.109375" customWidth="1"/>
+    <col min="16" max="16" width="31.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16" ht="25.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:16" ht="26.25" x14ac:dyDescent="0.25">
       <c r="B1" s="20" t="s">
         <v>0</v>
       </c>
@@ -1031,7 +1030,7 @@
       <c r="J1" s="21"/>
       <c r="K1" s="21"/>
     </row>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B2" s="22" t="s">
         <v>76</v>
       </c>
@@ -1045,7 +1044,7 @@
       <c r="J2" s="21"/>
       <c r="K2" s="21"/>
     </row>
-    <row r="4" spans="2:16" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:16" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
@@ -1082,7 +1081,7 @@
       <c r="O4" s="24"/>
       <c r="P4" s="24"/>
     </row>
-    <row r="5" spans="2:16" ht="90" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:16" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
         <v>10</v>
       </c>
@@ -1120,10 +1119,10 @@
       <c r="O5" s="25"/>
       <c r="P5" s="13">
         <f>COUNTIF($K$5:$K$148,"DECIDED")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:16" ht="201.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:16" ht="199.5" x14ac:dyDescent="0.25">
       <c r="B6" s="8" t="s">
         <v>17</v>
       </c>
@@ -1164,7 +1163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:16" ht="201.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:16" ht="199.5" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
         <v>18</v>
       </c>
@@ -1205,7 +1204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:16" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:16" ht="57" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
         <v>19</v>
       </c>
@@ -1243,10 +1242,10 @@
       <c r="O8" s="23"/>
       <c r="P8" s="14">
         <f>SUM(P5:P7)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
-    <row r="9" spans="2:16" ht="158.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:16" ht="156.75" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
         <v>24</v>
       </c>
@@ -1279,7 +1278,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="2:16" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:16" ht="42.75" x14ac:dyDescent="0.25">
       <c r="B10" s="8" t="s">
         <v>25</v>
       </c>
@@ -1312,7 +1311,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="2:16" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:16" ht="42.75" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
         <v>30</v>
       </c>
@@ -1345,7 +1344,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="12" spans="2:16" ht="72" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:16" ht="71.25" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
         <v>38</v>
       </c>
@@ -1378,7 +1377,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="2:16" ht="160.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:16" ht="160.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
         <v>47</v>
       </c>
@@ -1411,7 +1410,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="2:16" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:16" ht="150" x14ac:dyDescent="0.25">
       <c r="B14" s="7" t="s">
         <v>65</v>
       </c>
@@ -1444,7 +1443,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="2:16" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:16" ht="299.25" x14ac:dyDescent="0.25">
       <c r="B15" s="8" t="s">
         <v>78</v>
       </c>
@@ -1477,7 +1476,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="2:16" ht="316.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:16" ht="360" x14ac:dyDescent="0.25">
       <c r="B16" s="7" t="s">
         <v>79</v>
       </c>
@@ -1510,7 +1509,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="2:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:11" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="8" t="s">
         <v>88</v>
       </c>
@@ -1540,6 +1539,39 @@
         <v>15</v>
       </c>
       <c r="K17" s="12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11" ht="156.75" x14ac:dyDescent="0.25">
+      <c r="B18" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="C18" s="9">
+        <f>DATE(2026,9,29)</f>
+        <v>46294</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="F18" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="I18" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="J18" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="K18" s="12" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1554,77 +1586,72 @@
     <mergeCell ref="N7:O7"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
-  <conditionalFormatting sqref="C5:C12">
-    <cfRule type="cellIs" dxfId="16" priority="26" operator="equal">
-      <formula>"—"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C13">
-    <cfRule type="cellIs" dxfId="15" priority="22" operator="equal">
+  <conditionalFormatting sqref="C5:C13">
+    <cfRule type="cellIs" dxfId="13" priority="22" operator="equal">
       <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C15">
-    <cfRule type="cellIs" dxfId="14" priority="19" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="19" operator="equal">
+      <formula>"—"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C17:C18">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
       <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5">
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
       <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7">
-    <cfRule type="cellIs" dxfId="12" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="equal">
       <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9">
-    <cfRule type="cellIs" dxfId="11" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="4" operator="equal">
       <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="cellIs" dxfId="10" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="5" operator="equal">
       <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H16">
-    <cfRule type="cellIs" dxfId="8" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="7" operator="equal">
       <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J5">
-    <cfRule type="cellIs" dxfId="7" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="12" operator="equal">
       <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J11">
-    <cfRule type="cellIs" dxfId="6" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="11" operator="equal">
       <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J14">
-    <cfRule type="cellIs" dxfId="4" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="9" operator="equal">
       <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J16">
-    <cfRule type="cellIs" dxfId="3" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="8" operator="equal">
       <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:K17">
-    <cfRule type="containsText" dxfId="2" priority="23" operator="containsText" text="DECIDED">
+  <conditionalFormatting sqref="K5:K18">
+    <cfRule type="containsText" dxfId="1" priority="23" operator="containsText" text="DECIDED">
       <formula>NOT(ISERROR(SEARCH("DECIDED",K5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="24" operator="containsText" text="DEFERRED">
+    <cfRule type="containsText" dxfId="0" priority="24" operator="containsText" text="DEFERRED">
       <formula>NOT(ISERROR(SEARCH("DEFERRED",K5)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C17">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
-      <formula>"—"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>